<commit_message>
SEACAR DEV 0.7.0; update FigureCaptions; TrendText description updates
</commit_message>
<xml_diff>
--- a/inst/extdata/AtlasFigureCaptions_Final.xlsx
+++ b/inst/extdata/AtlasFigureCaptions_Final.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://floridadep.sharepoint.com/fco/seacar/seacar_expert_team/Shared Documents/SEACAR Website/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hill_T\Desktop\SEACAR GitHub\SEACAR-DEV\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{7FC53B06-1415-48DE-9F90-F745E0C275C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{712799C2-EA0C-4926-92B3-96A0298F43EE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8584E93-047F-4E25-B50B-E911AF75C76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$H$37</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="83">
   <si>
     <t>HabitatName</t>
   </si>
@@ -68,215 +68,233 @@
     <t>Percent Cover</t>
   </si>
   <si>
+    <t>Acreage</t>
+  </si>
+  <si>
+    <t>Hectares</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Acreage coverage maps of submerged aquatic vegetation. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Areal Extent</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Bar graph of the areal extent of submerged aquatic vegetation over time. Acreages from mapping efforts conducted at different resolutions, which are not always comparable, are graphed separately. Higher-resolution results are shown as blue open bars and lower-resolution results as green cross-hatched bars. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Water Column</t>
+  </si>
+  <si>
+    <t>Water Clarity</t>
+  </si>
+  <si>
+    <t>Chlorophyll a, Corrected for Pheophytin</t>
+  </si>
+  <si>
+    <t>Discrete</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average levels of chlorophyll a, corrected for pheophytin, over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only laboratory-analyzed chlorophyll a (triangles) is included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Chlorophyll a, Uncorrected for Pheophytin</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average levels of chlorophyll a, uncorrected for pheophytin, over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only laboratory-analyzed chlorophyll a (triangles) is included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Colored Dissolved Organic Matter</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average colored dissolved organic matter (CDOM) over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only laboratory-analyzed CDOM (triangles) is included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Water Quality</t>
+  </si>
+  <si>
+    <t>Dissolved Oxygen</t>
+  </si>
+  <si>
+    <t>Continuous</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only dissolved oxygen values measured in the field (circles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Dissolved Oxygen Saturation</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen saturation over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen saturation over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only dissolved oxygen saturation values measured in the field (circles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Salinity</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average salinity over time. If the time series included ten or more years of discrete observations, significant (blue) or non-significant (magenta) trend lines are also shown. Discrete salinity values derived from grab samples analyzed in the field (circles) or the laboratory (triangles) are both included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average salinity over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>pH</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average pH over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only pH values measured in the field (circles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average pH over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Water Temperature</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average water temperature over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average water temperature over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only water temperature measurements taken in the field (circles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Secchi Depth</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average Secchi depth over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Secchi depth is only measured in the field (circles).&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Turbidity</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average turbidity over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only turbidity values measured in the laboratory (triangles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average turbidity over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Nutrients</t>
+  </si>
+  <si>
+    <t>Total Nitrogen</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average total nitrogen over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only nitrogen values obtained from laboratory analyses (triangles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Total Phosphorus</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average total phosphorus over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only phosphorus values obtained from laboratory analyses (triangles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Total Suspended Solids</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average total suspended solids (TSS) over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only TSS values obtained from laboratory analyses (triangles) are included in the plot.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Nekton</t>
+  </si>
+  <si>
+    <t>Presence/Absence</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Bar graph(s) of annual average nekton richness over time for species groups occurring in at least 1% of samples. The bar colors represent species groups including bony fishes, cartilaginous fishes, decapod crustaceans (e.g., shrimps, crabs, and lobsters), and cephalopods (e.g., squid). Gear types and sizes are indicated in the panel label.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Oyster/Oyster Reef</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Acreage coverage maps of oyster reef. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Bar graph of the areal extent of oyster reefs over time. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Density</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of oyster density over time. If the time series included five or more years with observations, an estimated trend (blue line) and a 95% credible interval (purple band) may also be plotted. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Percent Live</t>
+  </si>
+  <si>
+    <t>Size Class</t>
+  </si>
+  <si>
+    <t>Shell Height</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plots of oyster sizes over time based on shells measuring at least 25 mm in height. A gray horizontal line at 75 mm marks the division between two size classes: 25 to 75 mm (circles) and greater than or equal to 75 mm (triangles). Estimated trends are shown as solid lines, and 95% credible intervals as shaded bands, for time series that included five or more years with observations. Shell heights of buried, dead oyster shells for which the years they lived were estimated (e.g., from calibrated radiocarbon results) are also shown in a separate plot, when available, to provide historical context. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Coastal Wetlands</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Acreage coverage maps of coastal wetlands. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Bar graph of the areal extent of coastal wetland types over time. These types include invasives (dark blue bars), mangroves (green), and/or marsh (blue). Acreages from mapping efforts conducted at different resolutions, which are not always comparable, are graphed separately. Higher-resolution results are shown as open bars and lower-resolution results as cross-hatched bars. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Species Composition</t>
+  </si>
+  <si>
+    <t>Total/Canopy Percent Cover</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Line graph of annual average coastal wetlands species richness over time for mangroves and associates (triangles), marsh (squares), and marsh succulents (circles). If the time series by species group included more than one year of observations, a line connects data points for visualization.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Coral/Coral Reef</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Acreage coverage maps of coral reefs. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Grazers and Reef Dependent Species</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Line graph of annual average species richness of grazers and reef-dependent species over time. If the time series included more than one year of observations, a line connects the data points for visualization.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of live coral coverage over time as a percent of reef surface. Species groups include octocorals, milleporans, and scleractinians. If the time series included five or more years of observations, a significant (blue) or non-significant (magenta) trend line is also shown. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Trend lines of median percent cover of submerged aquatic vegetation over time for species that had five or more years of observations. Line type represents significance (solid) or non-significance (dashed) of the trends.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of percent live oysters over time. If the time series included five or more years with observations, an estimated trend (blue line) and a 95% credible interval (purple band) may also be plotted. Estimation method is represented as percent (circles), point-intercept (triangle), or estimated percent (square), with data points jittered horizontally to reduce overlap.&lt;/p&gt;</t>
+  </si>
+  <si>
     <t>&lt;p&gt;Scatter plots of median percent cover of submerged aquatic vegetation over time by group. Plots for time series that included five or more years of observations show the estimated trend as a blue line.&lt;/p&gt;</t>
   </si>
   <si>
-    <t>Acreage</t>
-  </si>
-  <si>
-    <t>Hectares</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Acreage coverage maps of submerged aquatic vegetation. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Areal Extent</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Bar graph of the areal extent of submerged aquatic vegetation over time. Acreages from mapping efforts conducted at different resolutions, which are not always comparable, are graphed separately. Higher-resolution results are shown as blue open bars and lower-resolution results as green cross-hatched bars. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Water Column</t>
-  </si>
-  <si>
-    <t>Water Clarity</t>
-  </si>
-  <si>
-    <t>Chlorophyll a, Corrected for Pheophytin</t>
-  </si>
-  <si>
-    <t>Discrete</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average levels of chlorophyll a, corrected for pheophytin, over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only laboratory-analyzed chlorophyll a (triangles) is included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Chlorophyll a, Uncorrected for Pheophytin</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average levels of chlorophyll a, uncorrected for pheophytin, over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only laboratory-analyzed chlorophyll a (triangles) is included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Colored Dissolved Organic Matter</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average colored dissolved organic matter (CDOM) over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only laboratory-analyzed CDOM (triangles) is included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Water Quality</t>
-  </si>
-  <si>
-    <t>Dissolved Oxygen</t>
-  </si>
-  <si>
-    <t>Continuous</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only dissolved oxygen values measured in the field (circles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Dissolved Oxygen Saturation</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen saturation over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average dissolved oxygen saturation over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only dissolved oxygen saturation values measured in the field (circles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Salinity</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average salinity over time. If the time series included ten or more years of discrete observations, significant (blue) or non-significant (magenta) trend lines are also shown. Discrete salinity values derived from grab samples analyzed in the field (circles) or the laboratory (triangles) are both included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average salinity over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>pH</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average pH over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only pH values measured in the field (circles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average pH over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Water Temperature</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average water temperature over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average water temperature over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only water temperature measurements taken in the field (circles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Secchi Depth</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average Secchi depth over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Secchi depth is only measured in the field (circles).&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Turbidity</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average turbidity over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only turbidity values measured in the laboratory (triangles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average turbidity over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Nutrients</t>
-  </si>
-  <si>
-    <t>Total Nitrogen</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average total nitrogen over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only nitrogen values obtained from laboratory analyses (triangles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Total Phosphorus</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average total phosphorus over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only phosphorus values obtained from laboratory analyses (triangles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Total Suspended Solids</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of monthly average total suspended solids (TSS) over time. If the time series included ten or more years of discrete observations, a significant (blue) or non-significant (magenta) trend line is also shown. Only TSS values obtained from laboratory analyses (triangles) are included in the plot.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Nekton</t>
-  </si>
-  <si>
-    <t>Presence/Absence</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Bar graph(s) of annual average nekton richness over time for species groups occurring in at least 1% of samples. The bar colors represent species groups including bony fishes, cartilaginous fishes, decapod crustaceans (e.g., shrimps, crabs, and lobsters), and cephalopods (e.g., squid). Gear types and sizes are indicated in the panel label.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Oyster/Oyster Reef</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Acreage coverage maps of oyster reef. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Bar graph of the areal extent of oyster reefs over time. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Density</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of oyster density over time. If the time series included five or more years with observations, an estimated trend (blue line) and a 95% credible interval (purple band) may also be plotted. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Percent Live</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of percent live oysters over time. If the time series included five or more years with observations, an estimated trend (blue line) and a 95% credible interval (purple band) may also be plotted. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Size Class</t>
-  </si>
-  <si>
-    <t>Shell Height</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plots of oyster sizes over time based on shells measuring at least 25 mm in height. A gray horizontal line at 75 mm marks the division between two size classes: 25 to 75 mm (circles) and greater than or equal to 75 mm (triangles). Estimated trends are shown as solid lines, and 95% credible intervals as shaded bands, for time series that included five or more years with observations. Shell heights of buried, dead oyster shells for which the years they lived were estimated (e.g., from calibrated radiocarbon results) are also shown in a separate plot, when available, to provide historical context. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Coastal Wetlands</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Acreage coverage maps of coastal wetlands. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Bar graph of the areal extent of coastal wetland types over time. These types include invasives (dark blue bars), mangroves (green), and/or marsh (blue). Acreages from mapping efforts conducted at different resolutions, which are not always comparable, are graphed separately. Higher-resolution results are shown as open bars and lower-resolution results as cross-hatched bars. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Species Composition</t>
-  </si>
-  <si>
-    <t>Total/Canopy Percent Cover</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Line graph of annual average coastal wetlands species richness over time for mangroves and associates (triangles), marsh (squares), and marsh succulents (circles). If the time series by species group included more than one year of observations, a line connects data points for visualization.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Coral/Coral Reef</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Acreage coverage maps of coral reefs. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Grazers and Reef Dependent Species</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Line graph of annual average species richness of grazers and reef-dependent species over time. If the time series included more than one year of observations, a line connects the data points for visualization.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Scatter plot of live coral coverage over time as a percent of reef surface. Species groups include octocorals, milleporans, and scleractinians. If the time series included five or more years of observations, a significant (blue) or non-significant (magenta) trend line is also shown. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
+    <t>multiplot</t>
+  </si>
+  <si>
+    <t>trendplot</t>
+  </si>
+  <si>
+    <t>barplot</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Bar plot of submerged aquatic vegetation species occurrence frequency over time by group.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>PlotType</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -636,19 +654,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:H37"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
     <col min="3" max="3" width="28.140625" customWidth="1"/>
     <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="4" customWidth="1"/>
-    <col min="6" max="6" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1">
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -670,8 +688,11 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -685,694 +706,697 @@
         <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
       </c>
       <c r="E3" s="4">
         <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
       <c r="G4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
       </c>
       <c r="E5" s="4">
         <v>56</v>
       </c>
       <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
         <v>19</v>
       </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4">
         <v>25</v>
       </c>
       <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
-      </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" s="4">
         <v>29</v>
       </c>
       <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
         <v>23</v>
       </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>25</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
       </c>
       <c r="E8" s="4">
         <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E9" s="4">
         <v>40</v>
       </c>
       <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
         <v>28</v>
       </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" t="s">
-        <v>29</v>
-      </c>
       <c r="D10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" s="4">
         <v>45</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="4">
         <v>44</v>
       </c>
       <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E12" s="4">
         <v>52</v>
       </c>
       <c r="F12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
         <v>33</v>
       </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>26</v>
-      </c>
-      <c r="E13" s="4">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" t="s">
         <v>34</v>
       </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" t="s">
-        <v>35</v>
-      </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="4">
         <v>48</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E15" s="4">
         <v>49</v>
       </c>
       <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
         <v>37</v>
       </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
-      </c>
       <c r="D16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="4">
         <v>7</v>
       </c>
       <c r="F16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="4">
         <v>6</v>
       </c>
       <c r="F17" t="s">
+        <v>39</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" t="s">
         <v>40</v>
       </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" t="s">
-        <v>41</v>
-      </c>
       <c r="D18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E18" s="4">
         <v>31</v>
       </c>
       <c r="F18" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" t="s">
         <v>42</v>
       </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" t="s">
-        <v>43</v>
-      </c>
       <c r="D19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E19" s="4">
         <v>34</v>
       </c>
       <c r="F19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G19">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" t="s">
         <v>15</v>
       </c>
-      <c r="B20" t="s">
-        <v>16</v>
-      </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E20" s="4">
         <v>35</v>
       </c>
       <c r="F20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
         <v>45</v>
       </c>
-      <c r="G20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>46</v>
       </c>
-      <c r="C21" t="s">
-        <v>47</v>
-      </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E21" s="4">
         <v>21</v>
       </c>
       <c r="F21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" t="s">
         <v>48</v>
       </c>
-      <c r="G21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C22" t="s">
-        <v>49</v>
-      </c>
       <c r="D22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E22" s="4">
         <v>23</v>
       </c>
       <c r="F22" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
         <v>50</v>
       </c>
-      <c r="G22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
-        <v>15</v>
-      </c>
-      <c r="B23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23" t="s">
-        <v>51</v>
-      </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E23" s="4">
         <v>32</v>
       </c>
       <c r="F23" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
         <v>52</v>
       </c>
-      <c r="G23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>53</v>
-      </c>
-      <c r="C24" t="s">
-        <v>54</v>
       </c>
       <c r="E24" s="4">
         <v>53</v>
       </c>
       <c r="F24" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>55</v>
       </c>
-      <c r="G24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" t="s">
-        <v>56</v>
-      </c>
       <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
         <v>10</v>
-      </c>
-      <c r="C25" t="s">
-        <v>11</v>
       </c>
       <c r="E25" s="4">
         <v>15</v>
       </c>
       <c r="F25" t="s">
+        <v>56</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" t="s">
         <v>57</v>
       </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
         <v>58</v>
       </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" t="s">
-        <v>59</v>
-      </c>
       <c r="C27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E27" s="4">
         <v>16</v>
       </c>
       <c r="F27" t="s">
+        <v>59</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="G27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" t="s">
-        <v>61</v>
-      </c>
       <c r="C28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E28" s="4">
         <v>17</v>
       </c>
       <c r="F28" t="s">
+        <v>76</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" t="s">
         <v>62</v>
-      </c>
-      <c r="G28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" t="s">
-        <v>56</v>
-      </c>
-      <c r="B29" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" t="s">
-        <v>64</v>
       </c>
       <c r="E29" s="4">
         <v>18</v>
       </c>
       <c r="F29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G29">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
         <v>10</v>
-      </c>
-      <c r="C30" t="s">
-        <v>11</v>
       </c>
       <c r="E30" s="4">
         <v>10</v>
       </c>
       <c r="F30" t="s">
+        <v>65</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" t="s">
+        <v>66</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" t="s">
         <v>67</v>
       </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B31" t="s">
-        <v>13</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="C32" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" t="s">
-        <v>66</v>
-      </c>
-      <c r="B32" t="s">
-        <v>69</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="E32" s="4">
         <v>57</v>
       </c>
       <c r="F32" t="s">
+        <v>69</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="4">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
         <v>71</v>
       </c>
-      <c r="G32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" t="s">
+      <c r="G33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" t="s">
         <v>72</v>
       </c>
-      <c r="B33" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="4">
-        <v>14</v>
-      </c>
-      <c r="F33" t="s">
-        <v>73</v>
-      </c>
-      <c r="G33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" t="s">
-        <v>72</v>
-      </c>
-      <c r="B34" t="s">
-        <v>74</v>
-      </c>
       <c r="C34" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E34" s="4">
         <v>59</v>
       </c>
       <c r="F34" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
         <v>8</v>
@@ -1384,22 +1408,79 @@
         <v>58</v>
       </c>
       <c r="F35" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
     </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>77</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>81</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G35" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076DA15E4D2A7704AB61A56835D6241B7" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="abb5ff167b837d924831c3201942291d">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ed83551b-1c74-4eb0-a689-e3b00317a30f" xmlns:ns3="bb4cc7eb-2209-4410-ab26-7c1417e326d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cbd03875b41a39710f9853eeb0e782d3" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Version_x0020_of_x0020_Record xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">true</Version_x0020_of_x0020_Record>
+    <TaxCatchAll xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f" xsi:nil="true"/>
+    <_dlc_DocId xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">NPVFY6KNS3ZM-922007501-2304</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">
+      <Url>https://floridadep.sharepoint.com/fco/seacar/seacar_expert_team/_layouts/15/DocIdRedir.aspx?ID=NPVFY6KNS3ZM-922007501-2304</Url>
+      <Description>NPVFY6KNS3ZM-922007501-2304</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076DA15E4D2A7704AB61A56835D6241B7" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1cad8514759d78cefaf511642ee75763">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ed83551b-1c74-4eb0-a689-e3b00317a30f" xmlns:ns3="bb4cc7eb-2209-4410-ab26-7c1417e326d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0d82ed6cdea1ab3c0d6ccb26d453d6d9" ns2:_="" ns3:_="">
     <xsd:import namespace="ed83551b-1c74-4eb0-a689-e3b00317a30f"/>
     <xsd:import namespace="bb4cc7eb-2209-4410-ab26-7c1417e326d2"/>
     <xsd:element name="properties">
@@ -1437,7 +1518,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ed83551b-1c74-4eb0-a689-e3b00317a30f" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="_dlc_DocId" ma:index="8" nillable="true" ma:displayName="Document ID Value" ma:description="The value of the document ID assigned to this item." ma:internalName="_dlc_DocId" ma:readOnly="true">
+    <xsd:element name="_dlc_DocId" ma:index="8" nillable="true" ma:displayName="Document ID Value" ma:description="The value of the document ID assigned to this item." ma:indexed="true" ma:internalName="_dlc_DocId" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
@@ -1669,33 +1750,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Version_x0020_of_x0020_Record xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">true</Version_x0020_of_x0020_Record>
-    <TaxCatchAll xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f" xsi:nil="true"/>
-    <_dlc_DocId xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">NPVFY6KNS3ZM-922007501-2304</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">
-      <Url>https://floridadep.sharepoint.com/fco/seacar/seacar_expert_team/_layouts/15/DocIdRedir.aspx?ID=NPVFY6KNS3ZM-922007501-2304</Url>
-      <Description>NPVFY6KNS3ZM-922007501-2304</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -1745,18 +1800,63 @@
 </spe:Receivers>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E3E441-AE25-45BD-9B1B-B7CA1AB6D82C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{230CB5B1-A4D6-490A-9105-FA683D1B53FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bb4cc7eb-2209-4410-ab26-7c1417e326d2"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ed83551b-1c74-4eb0-a689-e3b00317a30f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{230CB5B1-A4D6-490A-9105-FA683D1B53FF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3CD6012-B59C-4A01-AD30-B4DAA48E93EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ed83551b-1c74-4eb0-a689-e3b00317a30f"/>
+    <ds:schemaRef ds:uri="bb4cc7eb-2209-4410-ab26-7c1417e326d2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A866A9A-190E-4E75-8B65-2013347B72B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22782C24-4120-4564-8BE9-E5DBC077CEBC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22782C24-4120-4564-8BE9-E5DBC077CEBC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A866A9A-190E-4E75-8B65-2013347B72B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
dead shell oyster descriptions; keep_na within clean_managed_areas
</commit_message>
<xml_diff>
--- a/inst/extdata/AtlasFigureCaptions_Final.xlsx
+++ b/inst/extdata/AtlasFigureCaptions_Final.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hill_T\Desktop\SEACAR GitHub\SEACAR-DEV\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8584E93-047F-4E25-B50B-E911AF75C76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEE1A75C-C556-4715-91D4-EBA5A849F8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$H$33</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="80">
   <si>
     <t>HabitatName</t>
   </si>
@@ -68,15 +68,9 @@
     <t>Percent Cover</t>
   </si>
   <si>
-    <t>Acreage</t>
-  </si>
-  <si>
     <t>Hectares</t>
   </si>
   <si>
-    <t>&lt;p&gt;Acreage coverage maps of submerged aquatic vegetation. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Areal Extent</t>
   </si>
   <si>
@@ -206,12 +200,6 @@
     <t>&lt;p&gt;Bar graph(s) of annual average nekton richness over time for species groups occurring in at least 1% of samples. The bar colors represent species groups including bony fishes, cartilaginous fishes, decapod crustaceans (e.g., shrimps, crabs, and lobsters), and cephalopods (e.g., squid). Gear types and sizes are indicated in the panel label.&lt;/p&gt;</t>
   </si>
   <si>
-    <t>Oyster/Oyster Reef</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Acreage coverage maps of oyster reef. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>&lt;p&gt;Bar graph of the areal extent of oyster reefs over time. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
   </si>
   <si>
@@ -230,15 +218,9 @@
     <t>Shell Height</t>
   </si>
   <si>
-    <t>&lt;p&gt;Scatter plots of oyster sizes over time based on shells measuring at least 25 mm in height. A gray horizontal line at 75 mm marks the division between two size classes: 25 to 75 mm (circles) and greater than or equal to 75 mm (triangles). Estimated trends are shown as solid lines, and 95% credible intervals as shaded bands, for time series that included five or more years with observations. Shell heights of buried, dead oyster shells for which the years they lived were estimated (e.g., from calibrated radiocarbon results) are also shown in a separate plot, when available, to provide historical context. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Coastal Wetlands</t>
   </si>
   <si>
-    <t>&lt;p&gt;Acreage coverage maps of coastal wetlands. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>&lt;p&gt;Bar graph of the areal extent of coastal wetland types over time. These types include invasives (dark blue bars), mangroves (green), and/or marsh (blue). Acreages from mapping efforts conducted at different resolutions, which are not always comparable, are graphed separately. Higher-resolution results are shown as open bars and lower-resolution results as cross-hatched bars. Monitoring programs providing acreage data are credited under the acreage map.&lt;/p&gt;</t>
   </si>
   <si>
@@ -251,12 +233,6 @@
     <t>&lt;p&gt;Line graph of annual average coastal wetlands species richness over time for mangroves and associates (triangles), marsh (squares), and marsh succulents (circles). If the time series by species group included more than one year of observations, a line connects data points for visualization.&lt;/p&gt;</t>
   </si>
   <si>
-    <t>Coral/Coral Reef</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Acreage coverage maps of coral reefs. Click the play button to view mapped habitat coverage over time.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Grazers and Reef Dependent Species</t>
   </si>
   <si>
@@ -288,6 +264,21 @@
   </si>
   <si>
     <t>PlotType</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plots of oyster sizes over time based on shells measuring at least 25mm in height. A gray horizontal line at 75mm marks the division between two size classes: 25 to 75mm (circles) and greater than or equal to 75mm (triangles). Estimated trends are shown as solid lines, and 95% credible intervals as shaded bands, for time series that included five or more years with observations. Shell heights of buried, dead oyster shells for which the years they lived were estimated (e.g., from calibrated radiocarbon results) are also shown in a separate plot, when available, to provide historical context. Data points are jittered horizontally to reduce overlap.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Oyster Reef</t>
+  </si>
+  <si>
+    <t>Coral Reef</t>
+  </si>
+  <si>
+    <t>Specific Conductivity</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Scatter plot of monthly average specific conductivity over time at continuously monitored program locations. Each location is analyzed separately, with significant (blue) or non-significant (magenta) trend lines shown for time series that included five or more years of observations.&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -654,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
@@ -662,7 +653,7 @@
     <col min="3" max="3" width="28.140625" customWidth="1"/>
     <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="4" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="6" max="6" width="255.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -689,7 +680,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -706,13 +697,13 @@
         <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -720,10 +711,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
       </c>
       <c r="E3" s="4">
         <v>19</v>
@@ -737,13 +728,22 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4">
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -751,19 +751,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
       <c r="E5" s="4">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
         <v>18</v>
@@ -774,19 +774,19 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E6" s="4">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
         <v>20</v>
@@ -797,22 +797,22 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E7" s="4">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -820,22 +820,22 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="4">
+        <v>40</v>
+      </c>
+      <c r="F8" t="s">
         <v>25</v>
-      </c>
-      <c r="E8" s="4">
-        <v>41</v>
-      </c>
-      <c r="F8" t="s">
-        <v>26</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -843,19 +843,19 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
-      </c>
       <c r="E9" s="4">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
         <v>27</v>
@@ -866,22 +866,22 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="4">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
         <v>28</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="4">
-        <v>45</v>
-      </c>
-      <c r="F10" t="s">
-        <v>29</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -889,19 +889,19 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E11" s="4">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="F11" t="s">
         <v>30</v>
@@ -912,22 +912,22 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
         <v>23</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E12" s="4">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
         <v>31</v>
-      </c>
-      <c r="D12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="4">
-        <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>32</v>
       </c>
       <c r="G12">
         <v>1</v>
@@ -935,19 +935,19 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E13" s="4">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
         <v>33</v>
@@ -958,22 +958,22 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
         <v>23</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" s="4">
+        <v>49</v>
+      </c>
+      <c r="F14" t="s">
         <v>34</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14" s="4">
-        <v>48</v>
-      </c>
-      <c r="F14" t="s">
-        <v>35</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -981,19 +981,19 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" t="s">
         <v>23</v>
       </c>
-      <c r="C15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" t="s">
-        <v>25</v>
-      </c>
       <c r="E15" s="4">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="F15" t="s">
         <v>36</v>
@@ -1004,42 +1004,42 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="4">
+        <v>6</v>
+      </c>
+      <c r="F16" t="s">
         <v>37</v>
       </c>
-      <c r="D16" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" s="4">
-        <v>7</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" t="s">
         <v>38</v>
       </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" t="s">
-        <v>37</v>
-      </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E17" s="4">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="F17" t="s">
         <v>39</v>
@@ -1048,21 +1048,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
         <v>40</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E18" s="4">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F18" t="s">
         <v>41</v>
@@ -1071,67 +1071,67 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="4">
+        <v>35</v>
+      </c>
+      <c r="F19" t="s">
+        <v>42</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
         <v>15</v>
       </c>
-      <c r="C19" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" t="s">
-        <v>17</v>
-      </c>
-      <c r="E19" s="4">
-        <v>34</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="E20" s="4">
+        <v>21</v>
+      </c>
+      <c r="F20" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
         <v>43</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B20" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" t="s">
-        <v>42</v>
-      </c>
-      <c r="D20" t="s">
-        <v>25</v>
-      </c>
-      <c r="E20" s="4">
-        <v>35</v>
-      </c>
-      <c r="F20" t="s">
-        <v>44</v>
-      </c>
-      <c r="G20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" t="s">
-        <v>45</v>
       </c>
       <c r="C21" t="s">
         <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E21" s="4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F21" t="s">
         <v>47</v>
@@ -1140,21 +1140,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
         <v>48</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E22" s="4">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F22" t="s">
         <v>49</v>
@@ -1163,135 +1163,138 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="E23" s="4">
+        <v>53</v>
+      </c>
+      <c r="F23" t="s">
+        <v>52</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="4">
         <v>15</v>
       </c>
-      <c r="C23" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="F24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" t="s">
+        <v>54</v>
+      </c>
+      <c r="E25" s="4">
+        <v>16</v>
+      </c>
+      <c r="F25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="4">
         <v>17</v>
       </c>
-      <c r="E23" s="4">
-        <v>32</v>
-      </c>
-      <c r="F23" t="s">
-        <v>51</v>
-      </c>
-      <c r="G23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B24" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" s="4">
-        <v>53</v>
-      </c>
-      <c r="F24" t="s">
-        <v>54</v>
-      </c>
-      <c r="G24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="4">
-        <v>15</v>
-      </c>
-      <c r="F25" t="s">
-        <v>56</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" t="s">
-        <v>12</v>
-      </c>
       <c r="F26" t="s">
+        <v>68</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" t="s">
         <v>57</v>
-      </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" t="s">
-        <v>58</v>
       </c>
       <c r="C27" t="s">
         <v>58</v>
       </c>
       <c r="E27" s="4">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s">
+        <v>75</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>59</v>
       </c>
-      <c r="G27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>55</v>
-      </c>
       <c r="B28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" s="4">
+        <v>10</v>
+      </c>
+      <c r="F28" t="s">
         <v>60</v>
       </c>
-      <c r="C28" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" s="4">
-        <v>17</v>
-      </c>
-      <c r="F28" t="s">
-        <v>76</v>
-      </c>
       <c r="G28">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B29" t="s">
         <v>61</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="1" t="s">
         <v>62</v>
       </c>
       <c r="E29" s="4">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="F29" t="s">
         <v>63</v>
@@ -1300,18 +1303,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" t="s">
         <v>64</v>
       </c>
-      <c r="B30" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" t="s">
-        <v>10</v>
+      <c r="C30" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="E30" s="4">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="F30" t="s">
         <v>65</v>
@@ -1320,12 +1323,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="4">
+        <v>58</v>
       </c>
       <c r="F31" t="s">
         <v>66</v>
@@ -1334,148 +1343,124 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="B32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E32" s="4">
-        <v>57</v>
+        <v>8</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
       </c>
       <c r="F32" t="s">
         <v>69</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F33" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H33" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>53</v>
+        <v>21</v>
+      </c>
+      <c r="C34" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" t="s">
+        <v>23</v>
       </c>
       <c r="E34" s="4">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F34" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>70</v>
-      </c>
-      <c r="B35" t="s">
-        <v>8</v>
-      </c>
-      <c r="C35" t="s">
-        <v>8</v>
-      </c>
-      <c r="E35" s="4">
-        <v>58</v>
-      </c>
-      <c r="F35" t="s">
-        <v>74</v>
-      </c>
-      <c r="G35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" t="s">
-        <v>8</v>
-      </c>
-      <c r="F36" t="s">
-        <v>77</v>
-      </c>
-      <c r="G36">
-        <v>0</v>
-      </c>
-      <c r="H36" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37" t="s">
-        <v>8</v>
-      </c>
-      <c r="C37" t="s">
-        <v>8</v>
-      </c>
-      <c r="F37" t="s">
-        <v>81</v>
-      </c>
-      <c r="G37">
-        <v>0</v>
-      </c>
-      <c r="H37" t="s">
-        <v>80</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H33" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Version_x0020_of_x0020_Record xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">true</Version_x0020_of_x0020_Record>
-    <TaxCatchAll xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f" xsi:nil="true"/>
-    <_dlc_DocId xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">NPVFY6KNS3ZM-922007501-2304</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">
-      <Url>https://floridadep.sharepoint.com/fco/seacar/seacar_expert_team/_layouts/15/DocIdRedir.aspx?ID=NPVFY6KNS3ZM-922007501-2304</Url>
-      <Description>NPVFY6KNS3ZM-922007501-2304</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1751,53 +1736,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Version_x0020_of_x0020_Record xmlns="bb4cc7eb-2209-4410-ab26-7c1417e326d2">true</Version_x0020_of_x0020_Record>
+    <TaxCatchAll xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f" xsi:nil="true"/>
+    <_dlc_DocId xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">NPVFY6KNS3ZM-922007501-2304</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="ed83551b-1c74-4eb0-a689-e3b00317a30f">
+      <Url>https://floridadep.sharepoint.com/fco/seacar/seacar_expert_team/_layouts/15/DocIdRedir.aspx?ID=NPVFY6KNS3ZM-922007501-2304</Url>
+      <Description>NPVFY6KNS3ZM-922007501-2304</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1810,18 +1762,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{230CB5B1-A4D6-490A-9105-FA683D1B53FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22782C24-4120-4564-8BE9-E5DBC077CEBC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="bb4cc7eb-2209-4410-ab26-7c1417e326d2"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ed83551b-1c74-4eb0-a689-e3b00317a30f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1846,9 +1789,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22782C24-4120-4564-8BE9-E5DBC077CEBC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{230CB5B1-A4D6-490A-9105-FA683D1B53FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bb4cc7eb-2209-4410-ab26-7c1417e326d2"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ed83551b-1c74-4eb0-a689-e3b00317a30f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>